<commit_message>
update skenario 22 sept
</commit_message>
<xml_diff>
--- a/LDC.xlsx
+++ b/LDC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/RegEco-PADAGIMO-SOLUSI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{0AE175BF-41C4-41B0-BB88-AEEA0AC58EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D55F7B5-0BEA-4FFC-8D23-DA1D8DACBC94}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{0AE175BF-41C4-41B0-BB88-AEEA0AC58EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC14C1C1-31D6-42C0-B38D-E603F1565F0F}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{381F0F33-FFEF-45E1-8129-DD167F3DDD36}"/>
   </bookViews>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="P6">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -1273,7 +1273,7 @@
         <v>0</v>
       </c>
       <c r="B7">
-        <v>2.5000000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -1294,13 +1294,13 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -1398,7 +1398,7 @@
         <v>0</v>
       </c>
       <c r="P8">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1463,7 +1463,7 @@
         <v>0</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="K9">
         <v>0</v>
@@ -1629,7 +1629,7 @@
         <v>0</v>
       </c>
       <c r="J11">
-        <v>0.5</v>
+        <v>0.92</v>
       </c>
       <c r="K11">
         <v>0</v>
@@ -1715,7 +1715,7 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>0.9</v>
+        <v>0.97</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -1875,7 +1875,7 @@
         <v>0</v>
       </c>
       <c r="I14">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -2065,13 +2065,13 @@
         <v>0</v>
       </c>
       <c r="Q16">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="R16">
         <v>0</v>
       </c>
       <c r="S16">
-        <v>0</v>
+        <v>1E-3</v>
       </c>
       <c r="T16">
         <v>0</v>
@@ -2148,7 +2148,7 @@
         <v>0</v>
       </c>
       <c r="Q17">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="R17">
         <v>0</v>
@@ -2183,7 +2183,7 @@
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="B18">
         <v>7.0000000000000007E-2</v>
@@ -2266,7 +2266,7 @@
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>0.19</v>
+        <v>0.03</v>
       </c>
       <c r="B19">
         <v>0.03</v>
@@ -2293,10 +2293,10 @@
         <v>0</v>
       </c>
       <c r="J19">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="K19">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L19">
         <v>0</v>
@@ -2317,7 +2317,7 @@
         <v>0</v>
       </c>
       <c r="R19">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="S19">
         <v>0</v>
@@ -2421,7 +2421,7 @@
         <v>0</v>
       </c>
       <c r="Y20">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="Z20">
         <v>0</v>
@@ -2444,11 +2444,11 @@
         <v>0</v>
       </c>
       <c r="E21">
+        <v>0.03</v>
+      </c>
+      <c r="F21">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F21">
-        <v>0.03</v>
-      </c>
       <c r="G21">
         <v>0</v>
       </c>
@@ -2492,13 +2492,13 @@
         <v>0</v>
       </c>
       <c r="U21">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="V21">
         <v>0</v>
       </c>
       <c r="W21">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="X21">
         <v>0</v>
@@ -2575,7 +2575,7 @@
         <v>0</v>
       </c>
       <c r="U22">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="V22">
         <v>0</v>
@@ -2658,10 +2658,10 @@
         <v>0</v>
       </c>
       <c r="U23">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="V23">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="W23">
         <v>0</v>
@@ -2821,7 +2821,7 @@
         <v>0</v>
       </c>
       <c r="T25">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="U25">
         <v>0</v>
@@ -2904,7 +2904,7 @@
         <v>0</v>
       </c>
       <c r="T26">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="U26">
         <v>0</v>
@@ -5835,79 +5835,79 @@
     </row>
     <row r="62" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>0.66</v>
+        <v>0.97</v>
       </c>
       <c r="B62">
-        <v>0.875</v>
+        <v>0.9</v>
       </c>
       <c r="C62">
         <v>1</v>
       </c>
       <c r="D62">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="E62">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="F62">
+        <v>0.92999999999999994</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62">
+        <v>0</v>
+      </c>
+      <c r="I62">
+        <v>0</v>
+      </c>
+      <c r="J62">
+        <v>0</v>
+      </c>
+      <c r="K62">
+        <v>0</v>
+      </c>
+      <c r="L62">
+        <v>0</v>
+      </c>
+      <c r="M62">
+        <v>0</v>
+      </c>
+      <c r="N62">
+        <v>0</v>
+      </c>
+      <c r="O62">
+        <v>0</v>
+      </c>
+      <c r="P62">
+        <v>0</v>
+      </c>
+      <c r="Q62">
+        <v>0.79</v>
+      </c>
+      <c r="R62">
         <v>0.97</v>
       </c>
-      <c r="G62">
-        <v>0</v>
-      </c>
-      <c r="H62">
-        <v>0</v>
-      </c>
-      <c r="I62">
-        <v>0.3</v>
-      </c>
-      <c r="J62">
-        <v>0.2</v>
-      </c>
-      <c r="K62">
-        <v>0</v>
-      </c>
-      <c r="L62">
-        <v>0</v>
-      </c>
-      <c r="M62">
-        <v>0</v>
-      </c>
-      <c r="N62">
-        <v>0</v>
-      </c>
-      <c r="O62">
-        <v>0</v>
-      </c>
-      <c r="P62">
-        <v>0.2</v>
-      </c>
-      <c r="Q62">
-        <v>0.7</v>
-      </c>
-      <c r="R62">
+      <c r="S62">
+        <v>0.999</v>
+      </c>
+      <c r="T62">
         <v>1</v>
       </c>
-      <c r="S62">
+      <c r="U62">
+        <v>0</v>
+      </c>
+      <c r="V62">
         <v>1</v>
       </c>
-      <c r="T62">
-        <v>0.2</v>
-      </c>
-      <c r="U62">
-        <v>0</v>
-      </c>
-      <c r="V62">
-        <v>0.5</v>
-      </c>
       <c r="W62">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="X62">
         <v>1</v>
       </c>
       <c r="Y62">
-        <v>0.67</v>
+        <v>0.8</v>
       </c>
       <c r="Z62">
         <v>1</v>

</xml_diff>